<commit_message>
daily auto-refresh 2026-08-05 18:01
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -468,9 +468,15 @@
       <c r="D2" t="n">
         <v>256</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>34</v>
+      </c>
+      <c r="F2" t="n">
+        <v>81</v>
+      </c>
+      <c r="G2" t="n">
+        <v>18012</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -487,9 +493,15 @@
       <c r="D3" t="n">
         <v>2677</v>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>297</v>
+      </c>
+      <c r="F3" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="G3" t="n">
+        <v>211765</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -506,9 +518,15 @@
       <c r="D4" t="n">
         <v>4047</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>387</v>
+      </c>
+      <c r="F4" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>41317</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -525,9 +543,15 @@
       <c r="D5" t="n">
         <v>4700</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>431</v>
+      </c>
+      <c r="F5" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>97276</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,9 +568,15 @@
       <c r="D6" t="n">
         <v>3294</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>314</v>
+      </c>
+      <c r="F6" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>53464</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -563,9 +593,15 @@
       <c r="D7" t="n">
         <v>6852</v>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>548</v>
+      </c>
+      <c r="F7" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>126265</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -582,9 +618,15 @@
       <c r="D8" t="n">
         <v>9880</v>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>786</v>
+      </c>
+      <c r="F8" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>86071</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -601,9 +643,15 @@
       <c r="D9" t="n">
         <v>11316</v>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>1280</v>
+      </c>
+      <c r="F9" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>165935</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -620,9 +668,15 @@
       <c r="D10" t="n">
         <v>6154</v>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>741</v>
+      </c>
+      <c r="F10" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>132896</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -639,9 +693,15 @@
       <c r="D11" t="n">
         <v>8747</v>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>514</v>
+      </c>
+      <c r="F11" t="n">
+        <v>61</v>
+      </c>
+      <c r="G11" t="n">
+        <v>42302</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -659,13 +719,13 @@
         <v>27744</v>
       </c>
       <c r="E12" t="n">
-        <v>1721</v>
+        <v>2149</v>
       </c>
       <c r="F12" t="n">
-        <v>47.4</v>
+        <v>59.2</v>
       </c>
       <c r="G12" t="n">
-        <v>30782</v>
+        <v>33437</v>
       </c>
     </row>
     <row r="13">
@@ -675,22 +735,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3054</v>
+        <v>3114</v>
       </c>
       <c r="C13" t="n">
-        <v>2338</v>
+        <v>2397</v>
       </c>
       <c r="D13" t="n">
-        <v>18186</v>
+        <v>18482</v>
       </c>
       <c r="E13" t="n">
-        <v>884</v>
+        <v>1036</v>
       </c>
       <c r="F13" t="n">
-        <v>37.8</v>
+        <v>43.2</v>
       </c>
       <c r="G13" t="n">
-        <v>21910</v>
+        <v>62243</v>
       </c>
     </row>
     <row r="14">
@@ -700,22 +760,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>192</v>
+        <v>265</v>
       </c>
       <c r="C14" t="n">
-        <v>79</v>
+        <v>140</v>
       </c>
       <c r="D14" t="n">
-        <v>1280</v>
+        <v>1636</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>8.9</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>242</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-07 14:17
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -525,7 +525,7 @@
         <v>63.8</v>
       </c>
       <c r="G4" t="n">
-        <v>41317</v>
+        <v>41367</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>59.9</v>
       </c>
       <c r="G5" t="n">
-        <v>97276</v>
+        <v>97491</v>
       </c>
     </row>
     <row r="6">
@@ -600,7 +600,7 @@
         <v>59.2</v>
       </c>
       <c r="G7" t="n">
-        <v>126265</v>
+        <v>126280</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>78.8</v>
       </c>
       <c r="G8" t="n">
-        <v>86071</v>
+        <v>86080</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>85.3</v>
       </c>
       <c r="G9" t="n">
-        <v>165935</v>
+        <v>166223</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         <v>87.90000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>132896</v>
+        <v>133045</v>
       </c>
     </row>
     <row r="11">
@@ -700,7 +700,7 @@
         <v>61</v>
       </c>
       <c r="G11" t="n">
-        <v>42302</v>
+        <v>42449</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +725,7 @@
         <v>59.2</v>
       </c>
       <c r="G12" t="n">
-        <v>33437</v>
+        <v>33534</v>
       </c>
     </row>
     <row r="13">
@@ -750,7 +750,7 @@
         <v>43.2</v>
       </c>
       <c r="G13" t="n">
-        <v>62243</v>
+        <v>62781</v>
       </c>
     </row>
     <row r="14">
@@ -760,13 +760,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>265</v>
+        <v>337</v>
       </c>
       <c r="C14" t="n">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="D14" t="n">
-        <v>1636</v>
+        <v>2038</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-08 14:15
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -650,7 +650,7 @@
         <v>85.3</v>
       </c>
       <c r="G9" t="n">
-        <v>166223</v>
+        <v>166248</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         <v>87.90000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>133045</v>
+        <v>133064</v>
       </c>
     </row>
     <row r="11">
@@ -700,7 +700,7 @@
         <v>61</v>
       </c>
       <c r="G11" t="n">
-        <v>42449</v>
+        <v>42459</v>
       </c>
     </row>
     <row r="12">
@@ -744,13 +744,13 @@
         <v>18482</v>
       </c>
       <c r="E13" t="n">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="F13" t="n">
-        <v>43.2</v>
+        <v>43.4</v>
       </c>
       <c r="G13" t="n">
-        <v>62781</v>
+        <v>62823</v>
       </c>
     </row>
     <row r="14">
@@ -760,13 +760,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>337</v>
+        <v>480</v>
       </c>
       <c r="C14" t="n">
-        <v>172</v>
+        <v>240</v>
       </c>
       <c r="D14" t="n">
-        <v>2038</v>
+        <v>2913</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -775,7 +775,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>222</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-11 14:16
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -500,7 +500,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>211765</v>
+        <v>211864</v>
       </c>
     </row>
     <row r="4">
@@ -525,7 +525,7 @@
         <v>63.8</v>
       </c>
       <c r="G4" t="n">
-        <v>41367</v>
+        <v>41430</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>59.9</v>
       </c>
       <c r="G5" t="n">
-        <v>97491</v>
+        <v>97800</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>63.6</v>
       </c>
       <c r="G6" t="n">
-        <v>53464</v>
+        <v>53493</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         <v>59.2</v>
       </c>
       <c r="G7" t="n">
-        <v>126280</v>
+        <v>126337</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>78.8</v>
       </c>
       <c r="G8" t="n">
-        <v>86080</v>
+        <v>86216</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>85.3</v>
       </c>
       <c r="G9" t="n">
-        <v>166248</v>
+        <v>168416</v>
       </c>
     </row>
     <row r="10">
@@ -669,13 +669,13 @@
         <v>6154</v>
       </c>
       <c r="E10" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="F10" t="n">
-        <v>87.90000000000001</v>
+        <v>88</v>
       </c>
       <c r="G10" t="n">
-        <v>133064</v>
+        <v>134610</v>
       </c>
     </row>
     <row r="11">
@@ -694,13 +694,13 @@
         <v>8747</v>
       </c>
       <c r="E11" t="n">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F11" t="n">
-        <v>61</v>
+        <v>61.2</v>
       </c>
       <c r="G11" t="n">
-        <v>42459</v>
+        <v>44803</v>
       </c>
     </row>
     <row r="12">
@@ -719,13 +719,13 @@
         <v>27744</v>
       </c>
       <c r="E12" t="n">
-        <v>2149</v>
+        <v>2157</v>
       </c>
       <c r="F12" t="n">
-        <v>59.2</v>
+        <v>59.4</v>
       </c>
       <c r="G12" t="n">
-        <v>33534</v>
+        <v>34234</v>
       </c>
     </row>
     <row r="13">
@@ -744,13 +744,13 @@
         <v>18482</v>
       </c>
       <c r="E13" t="n">
-        <v>1040</v>
+        <v>1091</v>
       </c>
       <c r="F13" t="n">
-        <v>43.4</v>
+        <v>45.5</v>
       </c>
       <c r="G13" t="n">
-        <v>62823</v>
+        <v>66015</v>
       </c>
     </row>
     <row r="14">
@@ -760,22 +760,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>528</v>
+        <v>620</v>
       </c>
       <c r="C14" t="n">
-        <v>265</v>
+        <v>294</v>
       </c>
       <c r="D14" t="n">
-        <v>3201</v>
+        <v>3643</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>12.6</v>
       </c>
       <c r="G14" t="n">
-        <v>298</v>
+        <v>621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix zeroed cost metrics and insights (None-safe sample-cost calc)
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -468,7 +468,7 @@
         <v>42</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="E2">
         <v>34</v>
@@ -491,7 +491,7 @@
         <v>436</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>2677</v>
       </c>
       <c r="E3">
         <v>297</v>
@@ -514,7 +514,7 @@
         <v>607</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>4047</v>
       </c>
       <c r="E4">
         <v>387</v>
@@ -537,7 +537,7 @@
         <v>719</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>4700</v>
       </c>
       <c r="E5">
         <v>431</v>
@@ -560,7 +560,7 @@
         <v>494</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>3294</v>
       </c>
       <c r="E6">
         <v>314</v>
@@ -583,7 +583,7 @@
         <v>925</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>6852</v>
       </c>
       <c r="E7">
         <v>548</v>
@@ -606,7 +606,7 @@
         <v>997</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>9880</v>
       </c>
       <c r="E8">
         <v>786</v>
@@ -629,7 +629,7 @@
         <v>1501</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>11316</v>
       </c>
       <c r="E9">
         <v>1280</v>
@@ -652,7 +652,7 @@
         <v>843</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>6154</v>
       </c>
       <c r="E10">
         <v>742</v>
@@ -675,7 +675,7 @@
         <v>842</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>8747</v>
       </c>
       <c r="E11">
         <v>515</v>
@@ -698,7 +698,7 @@
         <v>3631</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>27744</v>
       </c>
       <c r="E12">
         <v>2158</v>
@@ -721,7 +721,7 @@
         <v>2397</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>18482</v>
       </c>
       <c r="E13">
         <v>1098</v>
@@ -744,7 +744,7 @@
         <v>294</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>3643</v>
       </c>
       <c r="E14">
         <v>39</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-16 14:15
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -500,7 +500,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>212073</v>
+        <v>212295</v>
       </c>
     </row>
     <row r="4">
@@ -519,10 +519,10 @@
         <v>4047</v>
       </c>
       <c r="E4" t="n">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F4" t="n">
-        <v>63.8</v>
+        <v>63.6</v>
       </c>
       <c r="G4" t="n">
         <v>41469</v>
@@ -550,7 +550,7 @@
         <v>59.9</v>
       </c>
       <c r="G5" t="n">
-        <v>98118</v>
+        <v>98212</v>
       </c>
     </row>
     <row r="6">
@@ -563,7 +563,7 @@
         <v>534</v>
       </c>
       <c r="C6" t="n">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D6" t="n">
         <v>3294</v>
@@ -572,10 +572,10 @@
         <v>314</v>
       </c>
       <c r="F6" t="n">
-        <v>63.6</v>
+        <v>63.4</v>
       </c>
       <c r="G6" t="n">
-        <v>53550</v>
+        <v>53576</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         <v>59.2</v>
       </c>
       <c r="G7" t="n">
-        <v>126432</v>
+        <v>126444</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>78.90000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>86424</v>
+        <v>86546</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>85.3</v>
       </c>
       <c r="G9" t="n">
-        <v>169812</v>
+        <v>171088</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         <v>88</v>
       </c>
       <c r="G10" t="n">
-        <v>136253</v>
+        <v>136830</v>
       </c>
     </row>
     <row r="11">
@@ -688,7 +688,7 @@
         <v>1401</v>
       </c>
       <c r="C11" t="n">
-        <v>842</v>
+        <v>849</v>
       </c>
       <c r="D11" t="n">
         <v>8747</v>
@@ -697,10 +697,10 @@
         <v>515</v>
       </c>
       <c r="F11" t="n">
-        <v>61.2</v>
+        <v>60.7</v>
       </c>
       <c r="G11" t="n">
-        <v>47791</v>
+        <v>49247</v>
       </c>
     </row>
     <row r="12">
@@ -713,19 +713,19 @@
         <v>4459</v>
       </c>
       <c r="C12" t="n">
-        <v>3631</v>
+        <v>3634</v>
       </c>
       <c r="D12" t="n">
         <v>27744</v>
       </c>
       <c r="E12" t="n">
-        <v>2158</v>
+        <v>2160</v>
       </c>
       <c r="F12" t="n">
         <v>59.4</v>
       </c>
       <c r="G12" t="n">
-        <v>34937</v>
+        <v>35753</v>
       </c>
     </row>
     <row r="13">
@@ -738,19 +738,19 @@
         <v>3114</v>
       </c>
       <c r="C13" t="n">
-        <v>2400</v>
+        <v>2396</v>
       </c>
       <c r="D13" t="n">
         <v>18482</v>
       </c>
       <c r="E13" t="n">
-        <v>1103</v>
+        <v>1113</v>
       </c>
       <c r="F13" t="n">
-        <v>46</v>
+        <v>46.5</v>
       </c>
       <c r="G13" t="n">
-        <v>69320</v>
+        <v>70346</v>
       </c>
     </row>
     <row r="14">
@@ -760,22 +760,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>747</v>
+        <v>908</v>
       </c>
       <c r="C14" t="n">
-        <v>325</v>
+        <v>376</v>
       </c>
       <c r="D14" t="n">
-        <v>4329</v>
+        <v>5283</v>
       </c>
       <c r="E14" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="F14" t="n">
-        <v>14.2</v>
+        <v>15.4</v>
       </c>
       <c r="G14" t="n">
-        <v>892</v>
+        <v>1370</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-17 13:54
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -494,13 +494,13 @@
         <v>2677</v>
       </c>
       <c r="E3" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F3" t="n">
-        <v>68.09999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="G3" t="n">
-        <v>212295</v>
+        <v>212396</v>
       </c>
     </row>
     <row r="4">
@@ -525,7 +525,7 @@
         <v>63.6</v>
       </c>
       <c r="G4" t="n">
-        <v>41469</v>
+        <v>41510</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>59.9</v>
       </c>
       <c r="G5" t="n">
-        <v>98212</v>
+        <v>98295</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>63.4</v>
       </c>
       <c r="G6" t="n">
-        <v>53576</v>
+        <v>53591</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         <v>59.2</v>
       </c>
       <c r="G7" t="n">
-        <v>126444</v>
+        <v>126454</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>78.90000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>86546</v>
+        <v>86719</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>85.3</v>
       </c>
       <c r="G9" t="n">
-        <v>171088</v>
+        <v>173300</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         <v>88</v>
       </c>
       <c r="G10" t="n">
-        <v>136830</v>
+        <v>137993</v>
       </c>
     </row>
     <row r="11">
@@ -694,13 +694,13 @@
         <v>8747</v>
       </c>
       <c r="E11" t="n">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F11" t="n">
-        <v>60.7</v>
+        <v>60.8</v>
       </c>
       <c r="G11" t="n">
-        <v>49247</v>
+        <v>51181</v>
       </c>
     </row>
     <row r="12">
@@ -719,13 +719,13 @@
         <v>27744</v>
       </c>
       <c r="E12" t="n">
-        <v>2160</v>
+        <v>2161</v>
       </c>
       <c r="F12" t="n">
-        <v>59.4</v>
+        <v>59.5</v>
       </c>
       <c r="G12" t="n">
-        <v>35753</v>
+        <v>36732</v>
       </c>
     </row>
     <row r="13">
@@ -744,13 +744,13 @@
         <v>18482</v>
       </c>
       <c r="E13" t="n">
-        <v>1113</v>
+        <v>1118</v>
       </c>
       <c r="F13" t="n">
-        <v>46.5</v>
+        <v>46.7</v>
       </c>
       <c r="G13" t="n">
-        <v>70346</v>
+        <v>72031</v>
       </c>
     </row>
     <row r="14">
@@ -769,13 +769,13 @@
         <v>5283</v>
       </c>
       <c r="E14" t="n">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="F14" t="n">
-        <v>15.4</v>
+        <v>23.4</v>
       </c>
       <c r="G14" t="n">
-        <v>1370</v>
+        <v>1750</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-17 16:16
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -485,16 +485,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C3" t="n">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D3" t="n">
-        <v>2677</v>
+        <v>2671</v>
       </c>
       <c r="E3" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F3" t="n">
         <v>68.3</v>
@@ -510,22 +510,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>662</v>
+        <v>581</v>
       </c>
       <c r="C4" t="n">
-        <v>607</v>
+        <v>570</v>
       </c>
       <c r="D4" t="n">
-        <v>4047</v>
+        <v>3505</v>
       </c>
       <c r="E4" t="n">
-        <v>386</v>
+        <v>355</v>
       </c>
       <c r="F4" t="n">
-        <v>63.6</v>
+        <v>62.3</v>
       </c>
       <c r="G4" t="n">
-        <v>41510</v>
+        <v>37134</v>
       </c>
     </row>
     <row r="5">
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>765</v>
+        <v>640</v>
       </c>
       <c r="C5" t="n">
-        <v>719</v>
+        <v>630</v>
       </c>
       <c r="D5" t="n">
-        <v>4700</v>
+        <v>3862</v>
       </c>
       <c r="E5" t="n">
-        <v>431</v>
+        <v>355</v>
       </c>
       <c r="F5" t="n">
-        <v>59.9</v>
+        <v>56.3</v>
       </c>
       <c r="G5" t="n">
-        <v>98295</v>
+        <v>97010</v>
       </c>
     </row>
     <row r="6">
@@ -560,22 +560,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>534</v>
+        <v>436</v>
       </c>
       <c r="C6" t="n">
-        <v>495</v>
+        <v>431</v>
       </c>
       <c r="D6" t="n">
-        <v>3294</v>
+        <v>2638</v>
       </c>
       <c r="E6" t="n">
-        <v>314</v>
+        <v>259</v>
       </c>
       <c r="F6" t="n">
-        <v>63.4</v>
+        <v>60.1</v>
       </c>
       <c r="G6" t="n">
-        <v>53591</v>
+        <v>42387</v>
       </c>
     </row>
     <row r="7">
@@ -585,22 +585,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>979</v>
+        <v>838</v>
       </c>
       <c r="C7" t="n">
-        <v>925</v>
+        <v>815</v>
       </c>
       <c r="D7" t="n">
-        <v>6852</v>
+        <v>5545</v>
       </c>
       <c r="E7" t="n">
-        <v>548</v>
+        <v>462</v>
       </c>
       <c r="F7" t="n">
-        <v>59.2</v>
+        <v>56.7</v>
       </c>
       <c r="G7" t="n">
-        <v>126454</v>
+        <v>77391</v>
       </c>
     </row>
     <row r="8">
@@ -610,22 +610,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1113</v>
+        <v>883</v>
       </c>
       <c r="C8" t="n">
-        <v>997</v>
+        <v>822</v>
       </c>
       <c r="D8" t="n">
-        <v>9880</v>
+        <v>6624</v>
       </c>
       <c r="E8" t="n">
-        <v>787</v>
+        <v>647</v>
       </c>
       <c r="F8" t="n">
-        <v>78.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="G8" t="n">
-        <v>86719</v>
+        <v>85069</v>
       </c>
     </row>
     <row r="9">
@@ -635,22 +635,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1621</v>
+        <v>1545</v>
       </c>
       <c r="C9" t="n">
-        <v>1501</v>
+        <v>1489</v>
       </c>
       <c r="D9" t="n">
-        <v>11316</v>
+        <v>10168</v>
       </c>
       <c r="E9" t="n">
-        <v>1281</v>
+        <v>1272</v>
       </c>
       <c r="F9" t="n">
-        <v>85.3</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>173300</v>
+        <v>175572</v>
       </c>
     </row>
     <row r="10">
@@ -660,22 +660,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1000</v>
+        <v>993</v>
       </c>
       <c r="C10" t="n">
-        <v>843</v>
+        <v>878</v>
       </c>
       <c r="D10" t="n">
-        <v>6154</v>
+        <v>6031</v>
       </c>
       <c r="E10" t="n">
-        <v>742</v>
+        <v>776</v>
       </c>
       <c r="F10" t="n">
-        <v>88</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>137993</v>
+        <v>139204</v>
       </c>
     </row>
     <row r="11">
@@ -685,22 +685,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1401</v>
+        <v>1139</v>
       </c>
       <c r="C11" t="n">
-        <v>849</v>
+        <v>604</v>
       </c>
       <c r="D11" t="n">
-        <v>8747</v>
+        <v>6945</v>
       </c>
       <c r="E11" t="n">
-        <v>516</v>
+        <v>526</v>
       </c>
       <c r="F11" t="n">
-        <v>60.8</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>51181</v>
+        <v>52929</v>
       </c>
     </row>
     <row r="12">
@@ -710,22 +710,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4459</v>
+        <v>3817</v>
       </c>
       <c r="C12" t="n">
-        <v>3634</v>
+        <v>3044</v>
       </c>
       <c r="D12" t="n">
-        <v>27744</v>
+        <v>23443</v>
       </c>
       <c r="E12" t="n">
-        <v>2161</v>
+        <v>2191</v>
       </c>
       <c r="F12" t="n">
-        <v>59.5</v>
+        <v>72</v>
       </c>
       <c r="G12" t="n">
-        <v>36732</v>
+        <v>85297</v>
       </c>
     </row>
     <row r="13">
@@ -735,22 +735,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3114</v>
+        <v>3034</v>
       </c>
       <c r="C13" t="n">
-        <v>2396</v>
+        <v>2381</v>
       </c>
       <c r="D13" t="n">
-        <v>18482</v>
+        <v>17946</v>
       </c>
       <c r="E13" t="n">
-        <v>1118</v>
+        <v>1132</v>
       </c>
       <c r="F13" t="n">
-        <v>46.7</v>
+        <v>47.5</v>
       </c>
       <c r="G13" t="n">
-        <v>72031</v>
+        <v>72107</v>
       </c>
     </row>
     <row r="14">
@@ -760,22 +760,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1878</v>
+        <v>1794</v>
       </c>
       <c r="C14" t="n">
-        <v>657</v>
+        <v>612</v>
       </c>
       <c r="D14" t="n">
-        <v>10304</v>
+        <v>9741</v>
       </c>
       <c r="E14" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>14.6</v>
+        <v>16.3</v>
       </c>
       <c r="G14" t="n">
-        <v>25532</v>
+        <v>26987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add daily ethnicity mix table (date range + product filter)
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,111 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +113,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,377 +430,333 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>42</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>41</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>256</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>33</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>80.5</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>18012</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>441</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>435</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>2671</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>297</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>68.3</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>212426</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>581</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>570</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>3505</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>355</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>62.3</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>37169</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>640</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>630</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3862</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>355</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>56.3</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>97245</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>436</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>431</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>2638</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>259</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>60.1</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>42387</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>838</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>815</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>5545</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>462</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>56.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>77391</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>883</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>822</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>6624</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>647</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>78.7</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>85216</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>1545</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>1489</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>10168</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>1272</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>85.40000000000001</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>176347</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>993</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>878</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>6031</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>776</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>88.40000000000001</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>139806</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>1139</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>604</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>6945</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>527</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>87.3</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>53480</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>3817</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>3044</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>23443</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>2192</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>72</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>85570</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3034</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>2381</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>17946</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>1134</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>47.6</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>72394</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>1869</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>637</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>10123</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>131</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>20.6</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>27265</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-08-31 09:39
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -475,7 +475,7 @@
         <v>80.5</v>
       </c>
       <c r="G2" t="n">
-        <v>18063</v>
+        <v>18104</v>
       </c>
     </row>
     <row r="3">
@@ -500,7 +500,7 @@
         <v>68.3</v>
       </c>
       <c r="G3" t="n">
-        <v>212782</v>
+        <v>214085</v>
       </c>
     </row>
     <row r="4">
@@ -525,7 +525,7 @@
         <v>62.3</v>
       </c>
       <c r="G4" t="n">
-        <v>37338</v>
+        <v>37462</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>56.3</v>
       </c>
       <c r="G5" t="n">
-        <v>97863</v>
+        <v>98379</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>60.1</v>
       </c>
       <c r="G6" t="n">
-        <v>42597</v>
+        <v>42972</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         <v>56.7</v>
       </c>
       <c r="G7" t="n">
-        <v>77547</v>
+        <v>78043</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>78.8</v>
       </c>
       <c r="G8" t="n">
-        <v>86376</v>
+        <v>87583</v>
       </c>
     </row>
     <row r="9">
@@ -644,13 +644,13 @@
         <v>10168</v>
       </c>
       <c r="E9" t="n">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="F9" t="n">
-        <v>85.5</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>182587</v>
+        <v>188128</v>
       </c>
     </row>
     <row r="10">
@@ -669,13 +669,13 @@
         <v>6031</v>
       </c>
       <c r="E10" t="n">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="F10" t="n">
-        <v>88.40000000000001</v>
+        <v>88.5</v>
       </c>
       <c r="G10" t="n">
-        <v>142210</v>
+        <v>144087</v>
       </c>
     </row>
     <row r="11">
@@ -694,13 +694,13 @@
         <v>6945</v>
       </c>
       <c r="E11" t="n">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F11" t="n">
-        <v>87.3</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>58141</v>
+        <v>61365</v>
       </c>
     </row>
     <row r="12">
@@ -719,13 +719,13 @@
         <v>23443</v>
       </c>
       <c r="E12" t="n">
-        <v>2196</v>
+        <v>2193</v>
       </c>
       <c r="F12" t="n">
-        <v>72.09999999999999</v>
+        <v>72</v>
       </c>
       <c r="G12" t="n">
-        <v>88086</v>
+        <v>90488</v>
       </c>
     </row>
     <row r="13">
@@ -744,13 +744,13 @@
         <v>17946</v>
       </c>
       <c r="E13" t="n">
-        <v>1147</v>
+        <v>1157</v>
       </c>
       <c r="F13" t="n">
-        <v>48.2</v>
+        <v>48.6</v>
       </c>
       <c r="G13" t="n">
-        <v>76091</v>
+        <v>81052</v>
       </c>
     </row>
     <row r="14">
@@ -769,13 +769,13 @@
         <v>12657</v>
       </c>
       <c r="E14" t="n">
-        <v>292</v>
+        <v>370</v>
       </c>
       <c r="F14" t="n">
-        <v>35.3</v>
+        <v>44.7</v>
       </c>
       <c r="G14" t="n">
-        <v>30859</v>
+        <v>33637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-07 13:00
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -525,7 +525,7 @@
         <v>67.8</v>
       </c>
       <c r="G4" t="n">
-        <v>208360</v>
+        <v>208591</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>61.1</v>
       </c>
       <c r="G5" t="n">
-        <v>37612</v>
+        <v>38226</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>54.7</v>
       </c>
       <c r="G6" t="n">
-        <v>99160</v>
+        <v>99774</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         <v>59.9</v>
       </c>
       <c r="G7" t="n">
-        <v>43274</v>
+        <v>43326</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>55.5</v>
       </c>
       <c r="G8" t="n">
-        <v>78049</v>
+        <v>78201</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>77.2</v>
       </c>
       <c r="G9" t="n">
-        <v>79506</v>
+        <v>80753</v>
       </c>
     </row>
     <row r="10">
@@ -669,13 +669,13 @@
         <v>10168</v>
       </c>
       <c r="E10" t="n">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="F10" t="n">
-        <v>83.3</v>
+        <v>83.2</v>
       </c>
       <c r="G10" t="n">
-        <v>190202</v>
+        <v>191773</v>
       </c>
     </row>
     <row r="11">
@@ -700,7 +700,7 @@
         <v>86.7</v>
       </c>
       <c r="G11" t="n">
-        <v>144007</v>
+        <v>145524</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +725,7 @@
         <v>87.09999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>61233</v>
+        <v>62329</v>
       </c>
     </row>
     <row r="13">
@@ -750,7 +750,7 @@
         <v>69.7</v>
       </c>
       <c r="G13" t="n">
-        <v>88227</v>
+        <v>89264</v>
       </c>
     </row>
     <row r="14">
@@ -769,13 +769,13 @@
         <v>17922</v>
       </c>
       <c r="E14" t="n">
-        <v>1138</v>
+        <v>1140</v>
       </c>
       <c r="F14" t="n">
         <v>48.1</v>
       </c>
       <c r="G14" t="n">
-        <v>83697</v>
+        <v>85548</v>
       </c>
     </row>
     <row r="15">
@@ -794,13 +794,13 @@
         <v>13017</v>
       </c>
       <c r="E15" t="n">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="F15" t="n">
-        <v>46.5</v>
+        <v>47.1</v>
       </c>
       <c r="G15" t="n">
-        <v>35177</v>
+        <v>36275</v>
       </c>
     </row>
     <row r="16">
@@ -819,13 +819,13 @@
         <v>1588</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F16" t="n">
-        <v>6.8</v>
+        <v>21.2</v>
       </c>
       <c r="G16" t="n">
-        <v>199</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-08 14:08 (corrected 7 Sep GMV slabs)
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,117 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +119,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,427 +436,379 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>438</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>59</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>84.3</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>16791</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>256</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18104</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>441</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>432</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2671</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>294</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.09999999999999</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>208775</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>581</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>568</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3505</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>347</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>61.1</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>38346</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>640</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>629</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>3862</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>344</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>54.7</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>100162</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>436</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>431</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>2638</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>258</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>59.9</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>43326</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>838</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>811</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>5545</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>450</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>55.5</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>78236</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>883</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>821</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>6624</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>634</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>77.2</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>81069</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1545</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1486</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10168</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1238</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>83.3</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>192338</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>993</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>877</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>6031</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>760</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>86.7</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>146361</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1139</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>587</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6945</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>511</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>87.09999999999999</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>62747</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3814</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>3026</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>23425</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2109</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>69.7</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>89526</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>3030</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>2368</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>17922</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1138</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>48.1</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>85733</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2415</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>847</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>13017</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>399</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>47.1</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>36683</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>245</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>136</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>1640</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>40</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>29.4</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>396</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-09-09 13:01
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,117 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>sample_orders</t>
-  </si>
-  <si>
-    <t>new_creators</t>
-  </si>
-  <si>
-    <t>cogs</t>
-  </si>
-  <si>
-    <t>posted</t>
-  </si>
-  <si>
-    <t>post_rate</t>
-  </si>
-  <si>
-    <t>video_gmv</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-  <si>
-    <t>2026-04</t>
-  </si>
-  <si>
-    <t>2026-05</t>
-  </si>
-  <si>
-    <t>2026-06</t>
-  </si>
-  <si>
-    <t>2026-07</t>
-  </si>
-  <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>2026-09</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -119,36 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -436,379 +408,427 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sample_orders</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>new_creators</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cogs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>posted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>post_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>video_gmv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>73</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>70</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>438</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>59</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>84.3</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>16791</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>42</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>41</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>256</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>33</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>80.5</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>18104</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>441</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>432</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2671</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>294</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>68.09999999999999</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>208775</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>581</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>568</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3505</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>347</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>61.1</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>38346</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>640</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>629</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>3862</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>344</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>54.7</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>100162</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>436</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>431</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>2638</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>258</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>59.9</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>43326</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>838</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>811</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>5545</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>450</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>55.5</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>78236</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>883</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>821</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>6624</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>634</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>77.2</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>81069</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1545</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>1486</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>10168</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>1238</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>83.3</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>192338</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>993</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>877</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>6031</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>760</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>86.7</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>146361</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1139</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>587</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>6945</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>511</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>87.09999999999999</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>62747</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>3814</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>3026</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>23425</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>2109</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>69.7</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>89526</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>3030</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>2368</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>17922</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>1138</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>48.1</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>85733</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>2415</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="n">
         <v>847</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>13017</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>399</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>47.1</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>36683</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16">
-        <v>245</v>
-      </c>
-      <c r="C16">
-        <v>136</v>
-      </c>
-      <c r="D16">
-        <v>1640</v>
-      </c>
-      <c r="E16">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>294</v>
+      </c>
+      <c r="C16" t="n">
+        <v>150</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1936</v>
+      </c>
+      <c r="E16" t="n">
         <v>40</v>
       </c>
-      <c r="F16">
-        <v>29.4</v>
-      </c>
-      <c r="G16">
+      <c r="F16" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="G16" t="n">
         <v>396</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-09-11 15:01
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -525,7 +525,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>209128</v>
+        <v>209423</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>61.1</v>
       </c>
       <c r="G5" t="n">
-        <v>38744</v>
+        <v>38922</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>54.7</v>
       </c>
       <c r="G6" t="n">
-        <v>100631</v>
+        <v>100785</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         <v>59.9</v>
       </c>
       <c r="G7" t="n">
-        <v>43494</v>
+        <v>43545</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +625,7 @@
         <v>55.5</v>
       </c>
       <c r="G8" t="n">
-        <v>78352</v>
+        <v>78503</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         <v>77.2</v>
       </c>
       <c r="G9" t="n">
-        <v>81765</v>
+        <v>82383</v>
       </c>
     </row>
     <row r="10">
@@ -669,13 +669,13 @@
         <v>10168</v>
       </c>
       <c r="E10" t="n">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="F10" t="n">
-        <v>83.3</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>193358</v>
+        <v>193880</v>
       </c>
     </row>
     <row r="11">
@@ -700,7 +700,7 @@
         <v>86.7</v>
       </c>
       <c r="G11" t="n">
-        <v>147694</v>
+        <v>148165</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +725,7 @@
         <v>87.09999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>63744</v>
+        <v>63959</v>
       </c>
     </row>
     <row r="13">
@@ -744,13 +744,13 @@
         <v>23425</v>
       </c>
       <c r="E13" t="n">
-        <v>2107</v>
+        <v>2108</v>
       </c>
       <c r="F13" t="n">
-        <v>69.59999999999999</v>
+        <v>69.7</v>
       </c>
       <c r="G13" t="n">
-        <v>90547</v>
+        <v>90892</v>
       </c>
     </row>
     <row r="14">
@@ -769,13 +769,13 @@
         <v>17922</v>
       </c>
       <c r="E14" t="n">
-        <v>1138</v>
+        <v>1140</v>
       </c>
       <c r="F14" t="n">
         <v>48.1</v>
       </c>
       <c r="G14" t="n">
-        <v>87113</v>
+        <v>87490</v>
       </c>
     </row>
     <row r="15">
@@ -794,13 +794,13 @@
         <v>13017</v>
       </c>
       <c r="E15" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="F15" t="n">
-        <v>48.4</v>
+        <v>48.6</v>
       </c>
       <c r="G15" t="n">
-        <v>37549</v>
+        <v>37772</v>
       </c>
     </row>
     <row r="16">
@@ -819,13 +819,13 @@
         <v>2142</v>
       </c>
       <c r="E16" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F16" t="n">
-        <v>31.6</v>
+        <v>35.1</v>
       </c>
       <c r="G16" t="n">
-        <v>660</v>
+        <v>703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>